<commit_message>
feat: 支持 GitLab MR 统计并切换 CSV 导出
</commit_message>
<xml_diff>
--- a/output_demo.xlsx
+++ b/output_demo.xlsx
@@ -14,7 +14,6 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -34,54 +33,68 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
-  <si>
-    <t>时间</t>
-  </si>
-  <si>
-    <t>报告输出时间</t>
-  </si>
-  <si>
-    <t>xxx-xxxx-xxx xx：xx：xx</t>
-  </si>
-  <si>
-    <t>项目代码情况</t>
-  </si>
-  <si>
-    <t>人均生产力</t>
-  </si>
-  <si>
-    <t>项目名</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="15">
+  <si>
+    <t>时间：</t>
+  </si>
+  <si>
+    <t>开始时间</t>
+  </si>
+  <si>
+    <t>结束时间</t>
+  </si>
+  <si>
+    <t>项目代码变化情况</t>
+  </si>
+  <si>
+    <t>人均提交代码变化</t>
+  </si>
+  <si>
+    <t>项目名称</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>代码总行数</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>新增行数</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>删除行数</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>提交代码总行数</t>
-  </si>
-  <si>
-    <t>新增代码行数</t>
-  </si>
-  <si>
-    <t>删除代码行数</t>
-  </si>
-  <si>
-    <t>本周期提交人次</t>
-  </si>
-  <si>
-    <t>本周期人均提交代码行数</t>
-  </si>
-  <si>
-    <t>xxx-xxxx-xxx</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>本周期提交代码总行数</t>
-    <phoneticPr fontId="3" type="noConversion"/>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>提交次数</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>人均代码行数</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>姓名</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>提交总代码行</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>代码审核合格率</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -98,21 +111,26 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="0" tint="-4.9989318521683403E-2"/>
+      <sz val="9"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
+      <sz val="10.5"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10.5"/>
+      <color theme="1"/>
       <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -121,24 +139,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="-0.499984740745262"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="-0.249977111117893"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="5">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -198,45 +204,137 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -505,7 +603,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="21.26953125" customWidth="1"/>
@@ -516,137 +614,81 @@
     <col min="8" max="8" width="23.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:7" ht="14.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1" t="s">
+      <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="C1" s="8"/>
+      <c r="D1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="1"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
+    <row r="2" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="5" t="s">
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="6"/>
-      <c r="G2" s="7"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="5"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" s="3" t="s">
+      <c r="E3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="F3" s="1" t="s">
         <v>10</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="4"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="4"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="4"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="4"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="4"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="4"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="4"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="4"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A2:D2"/>
     <mergeCell ref="E2:G2"/>
-    <mergeCell ref="A2:D2"/>
   </mergeCells>
-  <phoneticPr fontId="3" type="noConversion"/>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -654,22 +696,68 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <phoneticPr fontId="3" type="noConversion"/>
+  <cols>
+    <col min="1" max="1" width="12.54296875" customWidth="1"/>
+    <col min="2" max="2" width="12.1796875" customWidth="1"/>
+    <col min="3" max="3" width="16.08984375" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="14.90625" customWidth="1"/>
+    <col min="7" max="7" width="20.26953125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="14.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="8"/>
+      <c r="D1" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="14.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="12"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <phoneticPr fontId="3" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>